<commit_message>
feat(seed): demo seeder — auth user, tenant, user_profile, 3 clients
Schema-aligned implementation of the Phase E plan Task 4. Diverges from
the plan in three ways (documented in module docstring):

- tenants.firm_name (plan said `name`); tenants.email is NOT NULL
- user_profiles (plural), keyed by id = auth.users.id, with full_name
- clients.entity_type 'company' (plan said 'private_limited' which fails
  the CHECK constraint)
- clients.fiscal_year_end is a single text column ('06-30')

Also fixes the fixture XLSX headers to match the parser's expected
"Taxable Amount (BDT)" / "VAT Amount (BDT)" labels (was missing parens),
and adds the missing fixtures package marker.

Verified end-to-end against the dev Supabase project: first run creates
everything, re-run logs `_exists` for every step.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/scripts/fixtures/demo_register.xlsx
+++ b/backend/scripts/fixtures/demo_register.xlsx
@@ -439,12 +439,12 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Taxable Amount BDT</t>
+          <t>Taxable Amount (BDT)</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>VAT Amount BDT</t>
+          <t>VAT Amount (BDT)</t>
         </is>
       </c>
     </row>

</xml_diff>